<commit_message>
Remove supplier branding from BOMs and CNC manufacturing files
</commit_message>
<xml_diff>
--- a/04_BOM/RP1_BOM_5DOF_MotionHead.xlsx
+++ b/04_BOM/RP1_BOM_5DOF_MotionHead.xlsx
@@ -404,7 +404,7 @@
     <t xml:space="preserve">模组</t>
   </si>
   <si>
-    <t xml:space="preserve">雷赛电机模组 PJ3-60CAN29</t>
+    <t xml:space="preserve">电机模组 PJ3-60CAN29</t>
   </si>
   <si>
     <t xml:space="preserve">YCL.E000084</t>
@@ -890,13 +890,13 @@
     <t xml:space="preserve">YCL.D000003</t>
   </si>
   <si>
-    <t xml:space="preserve">雷赛电机模组 PJ3-75CAN42</t>
+    <t xml:space="preserve">电机模组 PJ3-75CAN42</t>
   </si>
   <si>
     <t xml:space="preserve">YCL.D000001</t>
   </si>
   <si>
-    <t xml:space="preserve">雷赛电机模组 PJ3-97CAN140</t>
+    <t xml:space="preserve">电机模组 PJ3-97CAN140</t>
   </si>
   <si>
     <t xml:space="preserve">YCL.E000057</t>

</xml_diff>

<commit_message>
Apply approved motor model names and RP_Hand labels
</commit_message>
<xml_diff>
--- a/04_BOM/RP1_BOM_5DOF_MotionHead.xlsx
+++ b/04_BOM/RP1_BOM_5DOF_MotionHead.xlsx
@@ -404,7 +404,7 @@
     <t xml:space="preserve">模组</t>
   </si>
   <si>
-    <t xml:space="preserve">电机模组 PJ3-60CAN29</t>
+    <t xml:space="preserve">电机模组 RMM6562-2E</t>
   </si>
   <si>
     <t xml:space="preserve">YCL.E000084</t>
@@ -890,13 +890,13 @@
     <t xml:space="preserve">YCL.D000003</t>
   </si>
   <si>
-    <t xml:space="preserve">电机模组 PJ3-75CAN42</t>
+    <t xml:space="preserve">电机模组 RMM8463-2E</t>
   </si>
   <si>
     <t xml:space="preserve">YCL.D000001</t>
   </si>
   <si>
-    <t xml:space="preserve">电机模组 PJ3-97CAN140</t>
+    <t xml:space="preserve">电机模组 RMM10062-2E</t>
   </si>
   <si>
     <t xml:space="preserve">YCL.E000057</t>

</xml_diff>

<commit_message>
Synchronize motor part numbers with approved module catalog
</commit_message>
<xml_diff>
--- a/04_BOM/RP1_BOM_5DOF_MotionHead.xlsx
+++ b/04_BOM/RP1_BOM_5DOF_MotionHead.xlsx
@@ -398,7 +398,7 @@
     <t xml:space="preserve">轴承钢</t>
   </si>
   <si>
-    <t xml:space="preserve">YCL.D000002</t>
+    <t xml:space="preserve">YCL.D000020</t>
   </si>
   <si>
     <t xml:space="preserve">模组</t>
@@ -887,13 +887,13 @@
     <t xml:space="preserve">深沟球轴承61804-2RS</t>
   </si>
   <si>
-    <t xml:space="preserve">YCL.D000003</t>
+    <t xml:space="preserve">YCL.D000027</t>
   </si>
   <si>
     <t xml:space="preserve">电机模组 RMM8463-2E</t>
   </si>
   <si>
-    <t xml:space="preserve">YCL.D000001</t>
+    <t xml:space="preserve">YCL.D000031</t>
   </si>
   <si>
     <t xml:space="preserve">电机模组 RMM10062-2E</t>

</xml_diff>